<commit_message>
Added openpyxl scripting to create stacked bar chart of Gov't financing over past 6 years
</commit_message>
<xml_diff>
--- a/TT_Central_Gov_2026_Financing.xlsx
+++ b/TT_Central_Gov_2026_Financing.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Cen_GovTT_Financing" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TT_Gov_Borrowing" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -29,17 +29,19 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="13"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -51,8 +53,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F497D"/>
-        <bgColor rgb="001F497D"/>
+        <fgColor rgb="FF1F497D"/>
+        <bgColor rgb="FF1F497D"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +78,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -148,6 +150,218 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Central Government Gross Financing Architecture (TT$ Millions)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Cen_GovTT_Financing'!A5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2ECC71"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2ECC71"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cen_GovTT_Financing'!$B$1:$G$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cen_GovTT_Financing'!$B$5:$G$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Cen_GovTT_Financing'!A9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2980B9"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2980B9"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cen_GovTT_Financing'!$B$1:$G$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cen_GovTT_Financing'!$B$9:$G$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Cen_GovTT_Financing'!A4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="E67E22"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E67E22"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cen_GovTT_Financing'!$B$1:$G$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cen_GovTT_Financing'!$B$4:$G$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Financial Year Period</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Amount (TT$ Millions)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="$#,###.0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <absoluteAnchor>
+    <pos x="0" y="0"/>
+    <ext cx="0" cy="0"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </absoluteAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -440,19 +654,15 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="59" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="2" max="4"/>
+    <col width="21" customWidth="1" min="5" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr"/>
+    <row r="1" ht="17.4" customHeight="1">
+      <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Oct '20/
@@ -574,8 +784,8 @@
       <c r="B5" s="4" t="n">
         <v>6040.6</v>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n">
         <v>2495.6</v>
       </c>
@@ -642,12 +852,12 @@
           <t>of which:</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">

</xml_diff>